<commit_message>
Add basket price and checkout navigation tests
</commit_message>
<xml_diff>
--- a/src/test/java/test-cases-scenarios/Product-Test-Cases.xlsx
+++ b/src/test/java/test-cases-scenarios/Product-Test-Cases.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18192" windowHeight="6096"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -160,12 +161,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -180,9 +187,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -508,6 +516,7 @@
       <c r="C2" t="s">
         <v>39</v>
       </c>
+      <c r="F2" s="2"/>
       <c r="G2" t="s">
         <v>40</v>
       </c>
@@ -522,6 +531,7 @@
       <c r="C3" t="s">
         <v>39</v>
       </c>
+      <c r="F3" s="2"/>
       <c r="G3" t="s">
         <v>40</v>
       </c>
@@ -536,6 +546,7 @@
       <c r="C4" t="s">
         <v>39</v>
       </c>
+      <c r="F4" s="2"/>
       <c r="G4" t="s">
         <v>40</v>
       </c>
@@ -550,6 +561,7 @@
       <c r="C5" t="s">
         <v>39</v>
       </c>
+      <c r="F5" s="2"/>
       <c r="G5" t="s">
         <v>41</v>
       </c>
@@ -564,6 +576,7 @@
       <c r="C6" t="s">
         <v>39</v>
       </c>
+      <c r="F6" s="2"/>
       <c r="G6" t="s">
         <v>41</v>
       </c>
@@ -578,6 +591,7 @@
       <c r="C7" t="s">
         <v>39</v>
       </c>
+      <c r="F7" s="2"/>
       <c r="G7" t="s">
         <v>41</v>
       </c>
@@ -592,6 +606,7 @@
       <c r="C8" t="s">
         <v>39</v>
       </c>
+      <c r="F8" s="2"/>
       <c r="G8" t="s">
         <v>41</v>
       </c>
@@ -606,6 +621,7 @@
       <c r="C9" t="s">
         <v>39</v>
       </c>
+      <c r="F9" s="2"/>
       <c r="G9" t="s">
         <v>40</v>
       </c>
@@ -620,6 +636,7 @@
       <c r="C10" t="s">
         <v>39</v>
       </c>
+      <c r="F10" s="2"/>
       <c r="G10" t="s">
         <v>40</v>
       </c>
@@ -634,6 +651,7 @@
       <c r="C11" t="s">
         <v>39</v>
       </c>
+      <c r="F11" s="2"/>
       <c r="G11" t="s">
         <v>41</v>
       </c>
@@ -718,6 +736,7 @@
       <c r="C17" t="s">
         <v>39</v>
       </c>
+      <c r="F17" s="2"/>
       <c r="G17" t="s">
         <v>41</v>
       </c>

</xml_diff>